<commit_message>
zener added , doc updated
</commit_message>
<xml_diff>
--- a/OOP2025_Project_ScoresAllocation.xlsx
+++ b/OOP2025_Project_ScoresAllocation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arman\Documents\GitHub\OOP_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565191F6-58E5-4F28-84DE-C5E67794AA6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF603D6-368D-4338-8F0D-9ABEF6441378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
   <si>
     <t>عنوان</t>
   </si>
@@ -199,6 +199,9 @@
   </si>
   <si>
     <t>5?</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -577,22 +580,154 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="7" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="8" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -604,151 +739,19 @@
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -985,32 +988,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="24"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="75"/>
       <c r="J2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1019,17 +1022,17 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="62"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="37"/>
       <c r="J3" s="3">
         <v>5</v>
       </c>
@@ -1038,34 +1041,34 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="63" t="s">
+      <c r="A4" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="64"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="39"/>
       <c r="J4" s="3"/>
       <c r="K4" s="15"/>
     </row>
     <row r="5" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="65" t="s">
+      <c r="B5" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
-      <c r="H5" s="66"/>
-      <c r="I5" s="67"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="42"/>
       <c r="J5" s="3">
         <v>15</v>
       </c>
@@ -1074,17 +1077,17 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A6" s="21"/>
-      <c r="B6" s="32" t="s">
+      <c r="A6" s="47"/>
+      <c r="B6" s="43" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="34"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="45"/>
       <c r="J6" s="3">
         <v>15</v>
       </c>
@@ -1093,17 +1096,17 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A7" s="21"/>
-      <c r="B7" s="32" t="s">
+      <c r="A7" s="47"/>
+      <c r="B7" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="33"/>
-      <c r="I7" s="34"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="45"/>
       <c r="J7" s="4">
         <v>8</v>
       </c>
@@ -1112,17 +1115,17 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A8" s="21"/>
-      <c r="B8" s="32" t="s">
+      <c r="A8" s="47"/>
+      <c r="B8" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="34"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="45"/>
       <c r="J8" s="4">
         <v>10</v>
       </c>
@@ -1131,17 +1134,17 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="21"/>
-      <c r="B9" s="36" t="s">
+      <c r="A9" s="47"/>
+      <c r="B9" s="67" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="38"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="68"/>
+      <c r="F9" s="68"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="68"/>
+      <c r="I9" s="69"/>
       <c r="J9" s="5">
         <v>10</v>
       </c>
@@ -1150,36 +1153,36 @@
       </c>
     </row>
     <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A10" s="21"/>
-      <c r="B10" s="32" t="s">
+      <c r="A10" s="47"/>
+      <c r="B10" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="34"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="45"/>
       <c r="J10" s="4">
         <v>20</v>
       </c>
       <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="34"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="45"/>
       <c r="J11" s="4">
         <v>15</v>
       </c>
@@ -1188,51 +1191,55 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21"/>
-      <c r="B12" s="39" t="s">
+      <c r="A12" s="47"/>
+      <c r="B12" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="41"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="65"/>
+      <c r="F12" s="65"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
+      <c r="I12" s="66"/>
       <c r="J12" s="4">
         <v>15</v>
       </c>
-      <c r="K12" s="16"/>
+      <c r="K12" s="16">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A13" s="21"/>
-      <c r="B13" s="32" t="s">
+      <c r="A13" s="47"/>
+      <c r="B13" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="33"/>
-      <c r="I13" s="34"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="45"/>
       <c r="J13" s="6">
         <v>15</v>
       </c>
-      <c r="K13" s="15"/>
+      <c r="K13" s="15">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="21"/>
-      <c r="B14" s="39" t="s">
+      <c r="A14" s="47"/>
+      <c r="B14" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="41"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
+      <c r="I14" s="66"/>
       <c r="J14" s="6">
         <v>8</v>
       </c>
@@ -1241,34 +1248,36 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A15" s="21"/>
-      <c r="B15" s="32" t="s">
+      <c r="A15" s="47"/>
+      <c r="B15" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="33"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
-      <c r="I15" s="34"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="45"/>
       <c r="J15" s="6">
         <v>8</v>
       </c>
-      <c r="K15" s="15"/>
+      <c r="K15" s="15">
+        <v>8</v>
+      </c>
     </row>
     <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="21"/>
-      <c r="B16" s="39" t="s">
+      <c r="A16" s="47"/>
+      <c r="B16" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="41"/>
+      <c r="C16" s="65"/>
+      <c r="D16" s="65"/>
+      <c r="E16" s="65"/>
+      <c r="F16" s="65"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="65"/>
+      <c r="I16" s="66"/>
       <c r="J16" s="6">
         <v>15</v>
       </c>
@@ -1277,17 +1286,17 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="21"/>
-      <c r="B17" s="36" t="s">
+      <c r="A17" s="47"/>
+      <c r="B17" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="38"/>
+      <c r="C17" s="68"/>
+      <c r="D17" s="68"/>
+      <c r="E17" s="68"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="68"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="69"/>
       <c r="J17" s="5">
         <v>8</v>
       </c>
@@ -1296,68 +1305,74 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="21"/>
-      <c r="B18" s="36" t="s">
+      <c r="A18" s="47"/>
+      <c r="B18" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="38"/>
+      <c r="C18" s="68"/>
+      <c r="D18" s="68"/>
+      <c r="E18" s="68"/>
+      <c r="F18" s="68"/>
+      <c r="G18" s="68"/>
+      <c r="H18" s="68"/>
+      <c r="I18" s="69"/>
       <c r="J18" s="5">
         <v>12</v>
       </c>
-      <c r="K18" s="15"/>
+      <c r="K18" s="15">
+        <v>12</v>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="21"/>
-      <c r="B19" s="36" t="s">
+      <c r="A19" s="47"/>
+      <c r="B19" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="38"/>
+      <c r="C19" s="68"/>
+      <c r="D19" s="68"/>
+      <c r="E19" s="68"/>
+      <c r="F19" s="68"/>
+      <c r="G19" s="68"/>
+      <c r="H19" s="68"/>
+      <c r="I19" s="69"/>
       <c r="J19" s="5">
         <v>12</v>
       </c>
-      <c r="K19" s="15"/>
+      <c r="K19" s="15">
+        <v>12</v>
+      </c>
     </row>
     <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="21"/>
-      <c r="B20" s="36" t="s">
+      <c r="A20" s="47"/>
+      <c r="B20" s="67" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="37"/>
-      <c r="I20" s="38"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="68"/>
+      <c r="I20" s="69"/>
       <c r="J20" s="5">
         <v>5</v>
       </c>
-      <c r="K20" s="15"/>
+      <c r="K20" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="21"/>
-      <c r="B21" s="26" t="s">
+      <c r="A21" s="47"/>
+      <c r="B21" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="28"/>
+      <c r="C21" s="71"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="71"/>
+      <c r="F21" s="71"/>
+      <c r="G21" s="71"/>
+      <c r="H21" s="71"/>
+      <c r="I21" s="72"/>
       <c r="J21" s="5">
         <v>5</v>
       </c>
@@ -1366,53 +1381,53 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="21"/>
-      <c r="B22" s="29" t="s">
+      <c r="A22" s="47"/>
+      <c r="B22" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="31"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="62"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="63"/>
       <c r="J22" s="6">
         <v>7</v>
       </c>
       <c r="K22" s="15"/>
     </row>
     <row r="23" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="35"/>
-      <c r="B23" s="29" t="s">
+      <c r="A23" s="77"/>
+      <c r="B23" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="31"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
+      <c r="I23" s="63"/>
       <c r="J23" s="6">
         <v>12</v>
       </c>
       <c r="K23" s="15"/>
     </row>
     <row r="24" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="61" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="31"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
+      <c r="G24" s="62"/>
+      <c r="H24" s="62"/>
+      <c r="I24" s="63"/>
       <c r="J24" s="6">
         <v>10</v>
       </c>
@@ -1421,17 +1436,17 @@
       </c>
     </row>
     <row r="25" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="21"/>
-      <c r="B25" s="29" t="s">
+      <c r="A25" s="47"/>
+      <c r="B25" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="31"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="62"/>
+      <c r="H25" s="62"/>
+      <c r="I25" s="63"/>
       <c r="J25" s="6">
         <v>10</v>
       </c>
@@ -1440,17 +1455,17 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="21"/>
-      <c r="B26" s="29" t="s">
+      <c r="A26" s="47"/>
+      <c r="B26" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="31"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="62"/>
+      <c r="G26" s="62"/>
+      <c r="H26" s="62"/>
+      <c r="I26" s="63"/>
       <c r="J26" s="6">
         <v>20</v>
       </c>
@@ -1459,70 +1474,70 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="26" t="s">
+      <c r="A27" s="47"/>
+      <c r="B27" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="28"/>
+      <c r="C27" s="71"/>
+      <c r="D27" s="71"/>
+      <c r="E27" s="71"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="72"/>
       <c r="J27" s="5">
         <v>8</v>
       </c>
       <c r="K27" s="15"/>
     </row>
     <row r="28" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="21"/>
-      <c r="B28" s="26" t="s">
+      <c r="A28" s="47"/>
+      <c r="B28" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="28"/>
+      <c r="C28" s="71"/>
+      <c r="D28" s="71"/>
+      <c r="E28" s="71"/>
+      <c r="F28" s="71"/>
+      <c r="G28" s="71"/>
+      <c r="H28" s="71"/>
+      <c r="I28" s="72"/>
       <c r="J28" s="5">
         <v>15</v>
       </c>
       <c r="K28" s="15"/>
     </row>
     <row r="29" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="21"/>
-      <c r="B29" s="26" t="s">
+      <c r="A29" s="47"/>
+      <c r="B29" s="70" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="28"/>
+      <c r="C29" s="71"/>
+      <c r="D29" s="71"/>
+      <c r="E29" s="71"/>
+      <c r="F29" s="71"/>
+      <c r="G29" s="71"/>
+      <c r="H29" s="71"/>
+      <c r="I29" s="72"/>
       <c r="J29" s="5">
         <v>20</v>
       </c>
       <c r="K29" s="15"/>
     </row>
     <row r="30" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="49" t="s">
+      <c r="B30" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="50"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="50"/>
-      <c r="F30" s="50"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="50"/>
-      <c r="I30" s="51"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="57"/>
       <c r="J30" s="7">
         <v>8</v>
       </c>
@@ -1531,17 +1546,17 @@
       </c>
     </row>
     <row r="31" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="43"/>
-      <c r="B31" s="49" t="s">
+      <c r="A31" s="49"/>
+      <c r="B31" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="50"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="50"/>
-      <c r="F31" s="50"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="51"/>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
+      <c r="G31" s="56"/>
+      <c r="H31" s="56"/>
+      <c r="I31" s="57"/>
       <c r="J31" s="7">
         <v>8</v>
       </c>
@@ -1550,17 +1565,17 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="43"/>
-      <c r="B32" s="52" t="s">
+      <c r="A32" s="49"/>
+      <c r="B32" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="53"/>
-      <c r="F32" s="53"/>
-      <c r="G32" s="53"/>
-      <c r="H32" s="53"/>
-      <c r="I32" s="54"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="59"/>
+      <c r="I32" s="60"/>
       <c r="J32" s="8">
         <v>12</v>
       </c>
@@ -1569,208 +1584,210 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="43"/>
-      <c r="B33" s="52" t="s">
+      <c r="A33" s="49"/>
+      <c r="B33" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="C33" s="53"/>
-      <c r="D33" s="53"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="53"/>
-      <c r="G33" s="53"/>
-      <c r="H33" s="53"/>
-      <c r="I33" s="54"/>
+      <c r="C33" s="59"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="59"/>
+      <c r="H33" s="59"/>
+      <c r="I33" s="60"/>
       <c r="J33" s="8">
         <v>15</v>
       </c>
       <c r="K33" s="18"/>
     </row>
     <row r="34" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="43"/>
-      <c r="B34" s="49" t="s">
+      <c r="A34" s="49"/>
+      <c r="B34" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="50"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="50"/>
-      <c r="F34" s="50"/>
-      <c r="G34" s="50"/>
-      <c r="H34" s="50"/>
-      <c r="I34" s="51"/>
+      <c r="C34" s="56"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
+      <c r="G34" s="56"/>
+      <c r="H34" s="56"/>
+      <c r="I34" s="57"/>
       <c r="J34" s="7">
         <v>10</v>
       </c>
-      <c r="K34" s="17"/>
+      <c r="K34" s="17" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="35" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="43"/>
-      <c r="B35" s="49" t="s">
+      <c r="A35" s="49"/>
+      <c r="B35" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="50"/>
-      <c r="I35" s="51"/>
+      <c r="C35" s="56"/>
+      <c r="D35" s="56"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="56"/>
+      <c r="I35" s="57"/>
       <c r="J35" s="7">
         <v>10</v>
       </c>
       <c r="K35" s="17"/>
     </row>
     <row r="36" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="44" t="s">
+      <c r="A36" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="56"/>
-      <c r="I36" s="57"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="25"/>
       <c r="J36" s="9">
         <v>19</v>
       </c>
       <c r="K36" s="15"/>
     </row>
     <row r="37" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="45"/>
-      <c r="B37" s="55" t="s">
+      <c r="A37" s="51"/>
+      <c r="B37" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="C37" s="56"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="56"/>
-      <c r="H37" s="56"/>
-      <c r="I37" s="57"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="25"/>
       <c r="J37" s="9">
         <v>20</v>
       </c>
       <c r="K37" s="15"/>
     </row>
     <row r="38" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="45"/>
-      <c r="B38" s="55" t="s">
+      <c r="A38" s="51"/>
+      <c r="B38" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C38" s="56"/>
-      <c r="D38" s="56"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="56"/>
-      <c r="H38" s="56"/>
-      <c r="I38" s="57"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="24"/>
+      <c r="I38" s="25"/>
       <c r="J38" s="9">
         <v>30</v>
       </c>
       <c r="K38" s="15"/>
     </row>
     <row r="39" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="45"/>
-      <c r="B39" s="55" t="s">
+      <c r="A39" s="51"/>
+      <c r="B39" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="57"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="25"/>
       <c r="J39" s="9">
         <v>10</v>
       </c>
       <c r="K39" s="15"/>
     </row>
     <row r="40" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="45"/>
-      <c r="B40" s="58" t="s">
+      <c r="A40" s="51"/>
+      <c r="B40" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="59"/>
-      <c r="D40" s="59"/>
-      <c r="E40" s="59"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="59"/>
-      <c r="H40" s="59"/>
-      <c r="I40" s="60"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="28"/>
       <c r="J40" s="10">
         <v>10</v>
       </c>
       <c r="K40" s="15"/>
     </row>
     <row r="41" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="45"/>
-      <c r="B41" s="58" t="s">
+      <c r="A41" s="51"/>
+      <c r="B41" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="59"/>
-      <c r="D41" s="59"/>
-      <c r="E41" s="59"/>
-      <c r="F41" s="59"/>
-      <c r="G41" s="59"/>
-      <c r="H41" s="59"/>
-      <c r="I41" s="60"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="28"/>
       <c r="J41" s="10">
         <v>10</v>
       </c>
       <c r="K41" s="15"/>
     </row>
     <row r="42" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="45"/>
-      <c r="B42" s="58" t="s">
+      <c r="A42" s="51"/>
+      <c r="B42" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C42" s="59"/>
-      <c r="D42" s="59"/>
-      <c r="E42" s="59"/>
-      <c r="F42" s="59"/>
-      <c r="G42" s="59"/>
-      <c r="H42" s="59"/>
-      <c r="I42" s="60"/>
+      <c r="C42" s="27"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
+      <c r="I42" s="28"/>
       <c r="J42" s="10">
         <v>10</v>
       </c>
       <c r="K42" s="15"/>
     </row>
     <row r="43" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="46"/>
-      <c r="B43" s="71" t="s">
+      <c r="A43" s="52"/>
+      <c r="B43" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="C43" s="72"/>
-      <c r="D43" s="72"/>
-      <c r="E43" s="72"/>
-      <c r="F43" s="72"/>
-      <c r="G43" s="72"/>
-      <c r="H43" s="72"/>
-      <c r="I43" s="73"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
+      <c r="E43" s="30"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="31"/>
       <c r="J43" s="11">
         <v>5</v>
       </c>
       <c r="K43" s="16"/>
     </row>
     <row r="44" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="47" t="s">
+      <c r="A44" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="B44" s="74" t="s">
+      <c r="B44" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C44" s="75"/>
-      <c r="D44" s="75"/>
-      <c r="E44" s="75"/>
-      <c r="F44" s="75"/>
-      <c r="G44" s="75"/>
-      <c r="H44" s="75"/>
-      <c r="I44" s="76"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="33"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="33"/>
+      <c r="I44" s="34"/>
       <c r="J44" s="12">
         <v>15</v>
       </c>
@@ -1779,34 +1796,34 @@
       </c>
     </row>
     <row r="45" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="48"/>
-      <c r="B45" s="77" t="s">
+      <c r="A45" s="54"/>
+      <c r="B45" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C45" s="77"/>
-      <c r="D45" s="77"/>
-      <c r="E45" s="77"/>
-      <c r="F45" s="77"/>
-      <c r="G45" s="77"/>
-      <c r="H45" s="77"/>
-      <c r="I45" s="77"/>
+      <c r="C45" s="35"/>
+      <c r="D45" s="35"/>
+      <c r="E45" s="35"/>
+      <c r="F45" s="35"/>
+      <c r="G45" s="35"/>
+      <c r="H45" s="35"/>
+      <c r="I45" s="35"/>
       <c r="J45" s="12">
         <v>15</v>
       </c>
       <c r="K45" s="16"/>
     </row>
     <row r="46" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="48"/>
-      <c r="B46" s="77" t="s">
+      <c r="A46" s="54"/>
+      <c r="B46" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="C46" s="77"/>
-      <c r="D46" s="77"/>
-      <c r="E46" s="77"/>
-      <c r="F46" s="77"/>
-      <c r="G46" s="77"/>
-      <c r="H46" s="77"/>
-      <c r="I46" s="77"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="35"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="35"/>
+      <c r="I46" s="35"/>
       <c r="J46" s="12">
         <v>10</v>
       </c>
@@ -1818,19 +1835,19 @@
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
-      <c r="F47" s="68" t="s">
+      <c r="F47" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="G47" s="69"/>
-      <c r="H47" s="69"/>
-      <c r="I47" s="70"/>
+      <c r="G47" s="21"/>
+      <c r="H47" s="21"/>
+      <c r="I47" s="22"/>
       <c r="J47" s="13">
         <f>SUM(J3:J8, J10:J16, J22:J26, J30:J35, J36:J39)</f>
         <v>350</v>
       </c>
       <c r="K47" s="13">
         <f>SUM(K3:K8, K10:K16, K22:K26, K30:K35, K36:K39)</f>
-        <v>159</v>
+        <v>197</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -1839,19 +1856,19 @@
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
-      <c r="F48" s="68" t="s">
+      <c r="F48" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="G48" s="69"/>
-      <c r="H48" s="69"/>
-      <c r="I48" s="70"/>
+      <c r="G48" s="21"/>
+      <c r="H48" s="21"/>
+      <c r="I48" s="22"/>
       <c r="J48" s="13">
         <f>SUM(J9, J17:J21, J27:J29, J40:J43, J44:J46)</f>
         <v>170</v>
       </c>
       <c r="K48" s="13">
         <f>SUM(K9, K17:K21, K27:K29, K40:K43, K44:K46)</f>
-        <v>33</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -1860,19 +1877,19 @@
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
-      <c r="F49" s="68" t="s">
+      <c r="F49" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="G49" s="69"/>
-      <c r="H49" s="69"/>
-      <c r="I49" s="70"/>
+      <c r="G49" s="21"/>
+      <c r="H49" s="21"/>
+      <c r="I49" s="22"/>
       <c r="J49" s="13">
         <f>SUM(J3:J46)</f>
         <v>520</v>
       </c>
       <c r="K49" s="13">
         <f>SUM(K3:K46)</f>
-        <v>192</v>
+        <v>259</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1883,45 +1900,6 @@
     </row>
   </sheetData>
   <mergeCells count="55">
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B44:I44"/>
-    <mergeCell ref="B45:I45"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B39:I39"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="A5:A10"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="B17:I17"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B22:I22"/>
     <mergeCell ref="A24:A29"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A1:J1"/>
@@ -1938,6 +1916,45 @@
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B22:I22"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="A5:A10"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B39:I39"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
dependent sources added to cli
</commit_message>
<xml_diff>
--- a/OOP2025_Project_ScoresAllocation.xlsx
+++ b/OOP2025_Project_ScoresAllocation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arman\Documents\GitHub\OOP_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BCEF2D1-4320-4DA0-B114-A0D9018F7F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5E3EA29-9F11-4681-82C2-E2538731A307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -580,14 +580,110 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="7" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="8" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -605,27 +701,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -649,109 +724,34 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="7" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="8" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -989,32 +989,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="75"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="24"/>
       <c r="J2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1023,17 +1023,17 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="37"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="62"/>
       <c r="J3" s="3">
         <v>5</v>
       </c>
@@ -1042,34 +1042,34 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="63" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38"/>
-      <c r="H4" s="38"/>
-      <c r="I4" s="39"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="64"/>
       <c r="J4" s="3"/>
       <c r="K4" s="15"/>
     </row>
     <row r="5" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="42"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="67"/>
       <c r="J5" s="3">
         <v>15</v>
       </c>
@@ -1078,17 +1078,17 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A6" s="47"/>
-      <c r="B6" s="43" t="s">
+      <c r="A6" s="21"/>
+      <c r="B6" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="44"/>
-      <c r="H6" s="44"/>
-      <c r="I6" s="45"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="34"/>
       <c r="J6" s="3">
         <v>15</v>
       </c>
@@ -1097,17 +1097,17 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A7" s="47"/>
-      <c r="B7" s="43" t="s">
+      <c r="A7" s="21"/>
+      <c r="B7" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="45"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="34"/>
       <c r="J7" s="4">
         <v>8</v>
       </c>
@@ -1116,17 +1116,17 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A8" s="47"/>
-      <c r="B8" s="43" t="s">
+      <c r="A8" s="21"/>
+      <c r="B8" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="45"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="34"/>
       <c r="J8" s="4">
         <v>10</v>
       </c>
@@ -1135,17 +1135,17 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="47"/>
-      <c r="B9" s="67" t="s">
+      <c r="A9" s="21"/>
+      <c r="B9" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="68"/>
-      <c r="D9" s="68"/>
-      <c r="E9" s="68"/>
-      <c r="F9" s="68"/>
-      <c r="G9" s="68"/>
-      <c r="H9" s="68"/>
-      <c r="I9" s="69"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="38"/>
       <c r="J9" s="5">
         <v>10</v>
       </c>
@@ -1154,36 +1154,36 @@
       </c>
     </row>
     <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A10" s="47"/>
-      <c r="B10" s="43" t="s">
+      <c r="A10" s="21"/>
+      <c r="B10" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="45"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="34"/>
       <c r="J10" s="4">
         <v>20</v>
       </c>
       <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
-      <c r="I11" s="45"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="34"/>
       <c r="J11" s="4">
         <v>15</v>
       </c>
@@ -1192,17 +1192,17 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="47"/>
-      <c r="B12" s="64" t="s">
+      <c r="A12" s="21"/>
+      <c r="B12" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
-      <c r="I12" s="66"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="41"/>
       <c r="J12" s="4">
         <v>15</v>
       </c>
@@ -1211,17 +1211,17 @@
       </c>
     </row>
     <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A13" s="47"/>
-      <c r="B13" s="43" t="s">
+      <c r="A13" s="21"/>
+      <c r="B13" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="45"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="34"/>
       <c r="J13" s="6">
         <v>15</v>
       </c>
@@ -1230,17 +1230,17 @@
       </c>
     </row>
     <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="47"/>
-      <c r="B14" s="64" t="s">
+      <c r="A14" s="21"/>
+      <c r="B14" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="65"/>
-      <c r="D14" s="65"/>
-      <c r="E14" s="65"/>
-      <c r="F14" s="65"/>
-      <c r="G14" s="65"/>
-      <c r="H14" s="65"/>
-      <c r="I14" s="66"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="41"/>
       <c r="J14" s="6">
         <v>8</v>
       </c>
@@ -1249,17 +1249,17 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A15" s="47"/>
-      <c r="B15" s="43" t="s">
+      <c r="A15" s="21"/>
+      <c r="B15" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="45"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="34"/>
       <c r="J15" s="6">
         <v>8</v>
       </c>
@@ -1268,17 +1268,17 @@
       </c>
     </row>
     <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="47"/>
-      <c r="B16" s="64" t="s">
+      <c r="A16" s="21"/>
+      <c r="B16" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="65"/>
-      <c r="D16" s="65"/>
-      <c r="E16" s="65"/>
-      <c r="F16" s="65"/>
-      <c r="G16" s="65"/>
-      <c r="H16" s="65"/>
-      <c r="I16" s="66"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="41"/>
       <c r="J16" s="6">
         <v>15</v>
       </c>
@@ -1287,17 +1287,17 @@
       </c>
     </row>
     <row r="17" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="47"/>
-      <c r="B17" s="67" t="s">
+      <c r="A17" s="21"/>
+      <c r="B17" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="68"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="69"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="38"/>
       <c r="J17" s="5">
         <v>8</v>
       </c>
@@ -1306,17 +1306,17 @@
       </c>
     </row>
     <row r="18" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="47"/>
-      <c r="B18" s="67" t="s">
+      <c r="A18" s="21"/>
+      <c r="B18" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="68"/>
-      <c r="D18" s="68"/>
-      <c r="E18" s="68"/>
-      <c r="F18" s="68"/>
-      <c r="G18" s="68"/>
-      <c r="H18" s="68"/>
-      <c r="I18" s="69"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="38"/>
       <c r="J18" s="5">
         <v>12</v>
       </c>
@@ -1325,17 +1325,17 @@
       </c>
     </row>
     <row r="19" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="47"/>
-      <c r="B19" s="67" t="s">
+      <c r="A19" s="21"/>
+      <c r="B19" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="68"/>
-      <c r="D19" s="68"/>
-      <c r="E19" s="68"/>
-      <c r="F19" s="68"/>
-      <c r="G19" s="68"/>
-      <c r="H19" s="68"/>
-      <c r="I19" s="69"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="38"/>
       <c r="J19" s="5">
         <v>12</v>
       </c>
@@ -1344,17 +1344,17 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="47"/>
-      <c r="B20" s="67" t="s">
+      <c r="A20" s="21"/>
+      <c r="B20" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="68"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="68"/>
-      <c r="F20" s="68"/>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68"/>
-      <c r="I20" s="69"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="38"/>
       <c r="J20" s="5">
         <v>5</v>
       </c>
@@ -1363,17 +1363,17 @@
       </c>
     </row>
     <row r="21" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="47"/>
-      <c r="B21" s="70" t="s">
+      <c r="A21" s="21"/>
+      <c r="B21" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="71"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="71"/>
-      <c r="F21" s="71"/>
-      <c r="G21" s="71"/>
-      <c r="H21" s="71"/>
-      <c r="I21" s="72"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="28"/>
       <c r="J21" s="5">
         <v>5</v>
       </c>
@@ -1382,17 +1382,17 @@
       </c>
     </row>
     <row r="22" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="47"/>
-      <c r="B22" s="61" t="s">
+      <c r="A22" s="21"/>
+      <c r="B22" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="62"/>
-      <c r="D22" s="62"/>
-      <c r="E22" s="62"/>
-      <c r="F22" s="62"/>
-      <c r="G22" s="62"/>
-      <c r="H22" s="62"/>
-      <c r="I22" s="63"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="31"/>
       <c r="J22" s="6">
         <v>7</v>
       </c>
@@ -1401,17 +1401,17 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="77"/>
-      <c r="B23" s="61" t="s">
+      <c r="A23" s="35"/>
+      <c r="B23" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="62"/>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="62"/>
-      <c r="I23" s="63"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="31"/>
       <c r="J23" s="6">
         <v>12</v>
       </c>
@@ -1423,19 +1423,19 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="46" t="s">
+      <c r="A24" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="61" t="s">
+      <c r="B24" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="62"/>
-      <c r="H24" s="62"/>
-      <c r="I24" s="63"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="31"/>
       <c r="J24" s="6">
         <v>10</v>
       </c>
@@ -1444,17 +1444,17 @@
       </c>
     </row>
     <row r="25" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="47"/>
-      <c r="B25" s="61" t="s">
+      <c r="A25" s="21"/>
+      <c r="B25" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="62"/>
-      <c r="H25" s="62"/>
-      <c r="I25" s="63"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="31"/>
       <c r="J25" s="6">
         <v>10</v>
       </c>
@@ -1463,17 +1463,17 @@
       </c>
     </row>
     <row r="26" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="47"/>
-      <c r="B26" s="61" t="s">
+      <c r="A26" s="21"/>
+      <c r="B26" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="62"/>
-      <c r="H26" s="62"/>
-      <c r="I26" s="63"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="31"/>
       <c r="J26" s="6">
         <v>20</v>
       </c>
@@ -1482,70 +1482,72 @@
       </c>
     </row>
     <row r="27" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="47"/>
-      <c r="B27" s="70" t="s">
+      <c r="A27" s="21"/>
+      <c r="B27" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="71"/>
-      <c r="D27" s="71"/>
-      <c r="E27" s="71"/>
-      <c r="F27" s="71"/>
-      <c r="G27" s="71"/>
-      <c r="H27" s="71"/>
-      <c r="I27" s="72"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="28"/>
       <c r="J27" s="5">
         <v>8</v>
       </c>
       <c r="K27" s="15"/>
     </row>
     <row r="28" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="47"/>
-      <c r="B28" s="70" t="s">
+      <c r="A28" s="21"/>
+      <c r="B28" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="71"/>
-      <c r="D28" s="71"/>
-      <c r="E28" s="71"/>
-      <c r="F28" s="71"/>
-      <c r="G28" s="71"/>
-      <c r="H28" s="71"/>
-      <c r="I28" s="72"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="28"/>
       <c r="J28" s="5">
         <v>15</v>
       </c>
       <c r="K28" s="15"/>
     </row>
     <row r="29" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="47"/>
-      <c r="B29" s="70" t="s">
+      <c r="A29" s="21"/>
+      <c r="B29" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="71"/>
-      <c r="D29" s="71"/>
-      <c r="E29" s="71"/>
-      <c r="F29" s="71"/>
-      <c r="G29" s="71"/>
-      <c r="H29" s="71"/>
-      <c r="I29" s="72"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="28"/>
       <c r="J29" s="5">
         <v>20</v>
       </c>
-      <c r="K29" s="15"/>
+      <c r="K29" s="15">
+        <v>20</v>
+      </c>
     </row>
     <row r="30" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="48" t="s">
+      <c r="A30" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="55" t="s">
+      <c r="B30" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="56"/>
-      <c r="H30" s="56"/>
-      <c r="I30" s="57"/>
+      <c r="C30" s="50"/>
+      <c r="D30" s="50"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="50"/>
+      <c r="G30" s="50"/>
+      <c r="H30" s="50"/>
+      <c r="I30" s="51"/>
       <c r="J30" s="7">
         <v>8</v>
       </c>
@@ -1554,17 +1556,17 @@
       </c>
     </row>
     <row r="31" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="49"/>
-      <c r="B31" s="55" t="s">
+      <c r="A31" s="43"/>
+      <c r="B31" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="56"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="56"/>
-      <c r="F31" s="56"/>
-      <c r="G31" s="56"/>
-      <c r="H31" s="56"/>
-      <c r="I31" s="57"/>
+      <c r="C31" s="50"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="50"/>
+      <c r="G31" s="50"/>
+      <c r="H31" s="50"/>
+      <c r="I31" s="51"/>
       <c r="J31" s="7">
         <v>8</v>
       </c>
@@ -1573,17 +1575,17 @@
       </c>
     </row>
     <row r="32" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="49"/>
-      <c r="B32" s="58" t="s">
+      <c r="A32" s="43"/>
+      <c r="B32" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-      <c r="E32" s="59"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="59"/>
-      <c r="I32" s="60"/>
+      <c r="C32" s="53"/>
+      <c r="D32" s="53"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53"/>
+      <c r="G32" s="53"/>
+      <c r="H32" s="53"/>
+      <c r="I32" s="54"/>
       <c r="J32" s="8">
         <v>12</v>
       </c>
@@ -1592,17 +1594,17 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="49"/>
-      <c r="B33" s="58" t="s">
+      <c r="A33" s="43"/>
+      <c r="B33" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="59"/>
-      <c r="G33" s="59"/>
-      <c r="H33" s="59"/>
-      <c r="I33" s="60"/>
+      <c r="C33" s="53"/>
+      <c r="D33" s="53"/>
+      <c r="E33" s="53"/>
+      <c r="F33" s="53"/>
+      <c r="G33" s="53"/>
+      <c r="H33" s="53"/>
+      <c r="I33" s="54"/>
       <c r="J33" s="8">
         <v>15</v>
       </c>
@@ -1611,17 +1613,17 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="49"/>
-      <c r="B34" s="55" t="s">
+      <c r="A34" s="43"/>
+      <c r="B34" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="56"/>
-      <c r="I34" s="57"/>
+      <c r="C34" s="50"/>
+      <c r="D34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="50"/>
+      <c r="G34" s="50"/>
+      <c r="H34" s="50"/>
+      <c r="I34" s="51"/>
       <c r="J34" s="7">
         <v>10</v>
       </c>
@@ -1630,17 +1632,17 @@
       </c>
     </row>
     <row r="35" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="49"/>
-      <c r="B35" s="55" t="s">
+      <c r="A35" s="43"/>
+      <c r="B35" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="56"/>
-      <c r="D35" s="56"/>
-      <c r="E35" s="56"/>
-      <c r="F35" s="56"/>
-      <c r="G35" s="56"/>
-      <c r="H35" s="56"/>
-      <c r="I35" s="57"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+      <c r="E35" s="50"/>
+      <c r="F35" s="50"/>
+      <c r="G35" s="50"/>
+      <c r="H35" s="50"/>
+      <c r="I35" s="51"/>
       <c r="J35" s="7">
         <v>10</v>
       </c>
@@ -1649,157 +1651,157 @@
       </c>
     </row>
     <row r="36" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="50" t="s">
+      <c r="A36" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="23" t="s">
+      <c r="B36" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="25"/>
+      <c r="C36" s="56"/>
+      <c r="D36" s="56"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="56"/>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="57"/>
       <c r="J36" s="9">
         <v>19</v>
       </c>
       <c r="K36" s="15"/>
     </row>
     <row r="37" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="51"/>
-      <c r="B37" s="23" t="s">
+      <c r="A37" s="45"/>
+      <c r="B37" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="24"/>
-      <c r="I37" s="25"/>
+      <c r="C37" s="56"/>
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="57"/>
       <c r="J37" s="9">
         <v>20</v>
       </c>
       <c r="K37" s="15"/>
     </row>
     <row r="38" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="51"/>
-      <c r="B38" s="23" t="s">
+      <c r="A38" s="45"/>
+      <c r="B38" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="25"/>
+      <c r="C38" s="56"/>
+      <c r="D38" s="56"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="57"/>
       <c r="J38" s="9">
         <v>30</v>
       </c>
       <c r="K38" s="15"/>
     </row>
     <row r="39" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="51"/>
-      <c r="B39" s="23" t="s">
+      <c r="A39" s="45"/>
+      <c r="B39" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="24"/>
-      <c r="G39" s="24"/>
-      <c r="H39" s="24"/>
-      <c r="I39" s="25"/>
+      <c r="C39" s="56"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="57"/>
       <c r="J39" s="9">
         <v>10</v>
       </c>
       <c r="K39" s="15"/>
     </row>
     <row r="40" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="51"/>
-      <c r="B40" s="26" t="s">
+      <c r="A40" s="45"/>
+      <c r="B40" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="28"/>
+      <c r="C40" s="59"/>
+      <c r="D40" s="59"/>
+      <c r="E40" s="59"/>
+      <c r="F40" s="59"/>
+      <c r="G40" s="59"/>
+      <c r="H40" s="59"/>
+      <c r="I40" s="60"/>
       <c r="J40" s="10">
         <v>10</v>
       </c>
       <c r="K40" s="15"/>
     </row>
     <row r="41" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="51"/>
-      <c r="B41" s="26" t="s">
+      <c r="A41" s="45"/>
+      <c r="B41" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="28"/>
+      <c r="C41" s="59"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="59"/>
+      <c r="F41" s="59"/>
+      <c r="G41" s="59"/>
+      <c r="H41" s="59"/>
+      <c r="I41" s="60"/>
       <c r="J41" s="10">
         <v>10</v>
       </c>
       <c r="K41" s="15"/>
     </row>
     <row r="42" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="51"/>
-      <c r="B42" s="26" t="s">
+      <c r="A42" s="45"/>
+      <c r="B42" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="C42" s="27"/>
-      <c r="D42" s="27"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="27"/>
-      <c r="I42" s="28"/>
+      <c r="C42" s="59"/>
+      <c r="D42" s="59"/>
+      <c r="E42" s="59"/>
+      <c r="F42" s="59"/>
+      <c r="G42" s="59"/>
+      <c r="H42" s="59"/>
+      <c r="I42" s="60"/>
       <c r="J42" s="10">
         <v>10</v>
       </c>
       <c r="K42" s="15"/>
     </row>
     <row r="43" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="52"/>
-      <c r="B43" s="29" t="s">
+      <c r="A43" s="46"/>
+      <c r="B43" s="71" t="s">
         <v>30</v>
       </c>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
-      <c r="F43" s="30"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="30"/>
-      <c r="I43" s="31"/>
+      <c r="C43" s="72"/>
+      <c r="D43" s="72"/>
+      <c r="E43" s="72"/>
+      <c r="F43" s="72"/>
+      <c r="G43" s="72"/>
+      <c r="H43" s="72"/>
+      <c r="I43" s="73"/>
       <c r="J43" s="11">
         <v>5</v>
       </c>
       <c r="K43" s="16"/>
     </row>
     <row r="44" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="53" t="s">
+      <c r="A44" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="B44" s="32" t="s">
+      <c r="B44" s="74" t="s">
         <v>41</v>
       </c>
-      <c r="C44" s="33"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="33"/>
-      <c r="G44" s="33"/>
-      <c r="H44" s="33"/>
-      <c r="I44" s="34"/>
+      <c r="C44" s="75"/>
+      <c r="D44" s="75"/>
+      <c r="E44" s="75"/>
+      <c r="F44" s="75"/>
+      <c r="G44" s="75"/>
+      <c r="H44" s="75"/>
+      <c r="I44" s="76"/>
       <c r="J44" s="12">
         <v>15</v>
       </c>
@@ -1808,34 +1810,34 @@
       </c>
     </row>
     <row r="45" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="54"/>
-      <c r="B45" s="35" t="s">
+      <c r="A45" s="48"/>
+      <c r="B45" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="C45" s="35"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="35"/>
-      <c r="F45" s="35"/>
-      <c r="G45" s="35"/>
-      <c r="H45" s="35"/>
-      <c r="I45" s="35"/>
+      <c r="C45" s="77"/>
+      <c r="D45" s="77"/>
+      <c r="E45" s="77"/>
+      <c r="F45" s="77"/>
+      <c r="G45" s="77"/>
+      <c r="H45" s="77"/>
+      <c r="I45" s="77"/>
       <c r="J45" s="12">
         <v>15</v>
       </c>
       <c r="K45" s="16"/>
     </row>
     <row r="46" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="54"/>
-      <c r="B46" s="35" t="s">
+      <c r="A46" s="48"/>
+      <c r="B46" s="77" t="s">
         <v>43</v>
       </c>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="35"/>
+      <c r="C46" s="77"/>
+      <c r="D46" s="77"/>
+      <c r="E46" s="77"/>
+      <c r="F46" s="77"/>
+      <c r="G46" s="77"/>
+      <c r="H46" s="77"/>
+      <c r="I46" s="77"/>
       <c r="J46" s="12">
         <v>10</v>
       </c>
@@ -1847,12 +1849,12 @@
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
-      <c r="F47" s="20" t="s">
+      <c r="F47" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="G47" s="21"/>
-      <c r="H47" s="21"/>
-      <c r="I47" s="22"/>
+      <c r="G47" s="69"/>
+      <c r="H47" s="69"/>
+      <c r="I47" s="70"/>
       <c r="J47" s="13">
         <f>SUM(J3:J8, J10:J16, J22:J26, J30:J35, J36:J39)</f>
         <v>350</v>
@@ -1868,19 +1870,19 @@
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
-      <c r="F48" s="20" t="s">
+      <c r="F48" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="G48" s="21"/>
-      <c r="H48" s="21"/>
-      <c r="I48" s="22"/>
+      <c r="G48" s="69"/>
+      <c r="H48" s="69"/>
+      <c r="I48" s="70"/>
       <c r="J48" s="13">
         <f>SUM(J9, J17:J21, J27:J29, J40:J43, J44:J46)</f>
         <v>170</v>
       </c>
       <c r="K48" s="13">
         <f>SUM(K9, K17:K21, K27:K29, K40:K43, K44:K46)</f>
-        <v>62</v>
+        <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -1889,19 +1891,19 @@
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
-      <c r="F49" s="20" t="s">
+      <c r="F49" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="G49" s="21"/>
-      <c r="H49" s="21"/>
-      <c r="I49" s="22"/>
+      <c r="G49" s="69"/>
+      <c r="H49" s="69"/>
+      <c r="I49" s="70"/>
       <c r="J49" s="13">
         <f>SUM(J3:J46)</f>
         <v>520</v>
       </c>
       <c r="K49" s="13">
         <f>SUM(K3:K46)</f>
-        <v>307</v>
+        <v>327</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1912,6 +1914,45 @@
     </row>
   </sheetData>
   <mergeCells count="55">
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="A5:A10"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B22:I22"/>
     <mergeCell ref="A24:A29"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A1:J1"/>
@@ -1928,45 +1969,6 @@
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="B18:I18"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="B17:I17"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B22:I22"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="A5:A10"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B44:I44"/>
-    <mergeCell ref="B45:I45"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B39:I39"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>